<commit_message>
added a formula for all score rows or the column of scores but it has a bug where each input has space above and below
</commit_message>
<xml_diff>
--- a/student_scores.xlsx
+++ b/student_scores.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -445,63 +445,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>wefwe</t>
+          <t>waef</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>You Need To Study More</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>hrtrt</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>79</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>hrta</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>84</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>joshua</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>97</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-    </row>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -510,28 +469,6 @@
       </c>
       <c r="B7">
         <f>AVERAGE(B2:B5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Average</t>
-        </is>
-      </c>
-      <c r="B9">
-        <f>AVERAGE(B2:B7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Average</t>
-        </is>
-      </c>
-      <c r="B11">
-        <f>AVERAGE(B2:B9)</f>
         <v/>
       </c>
     </row>

</xml_diff>